<commit_message>
Bao gia PR quoc te: ghi ro chinh sach bao hanh, site le, VAT (Hieu 30/10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-PR-Quoc-Te-Nha-Khoa-2026-10-30.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-PR-Quoc-Te-Nha-Khoa-2026-10-30.xlsx
@@ -629,7 +629,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Các bước triển khai, nội dung, bảo hành, hoá đơn</t>
+          <t>Chính sách nội dung, thời gian, bảo hành, hoá đơn và các bước triển khai</t>
         </is>
       </c>
     </row>
@@ -649,10 +649,10 @@
       </c>
     </row>
     <row r="9"/>
-    <row r="10" ht="34" customHeight="1">
+    <row r="10" ht="52" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Giá tính bằng VNĐ, đơn hàng PR quốc tế không xuất hoá đơn VAT. Giá ưu đãi là giá thanh toán.</t>
+          <t>Giá tính bằng VNĐ, giá ưu đãi là giá thanh toán. Đơn hàng PR quốc tế KHÔNG xuất hoá đơn VAT. Bảo hành 03 tháng: bài bị gỡ được đăng lại miễn phí. Đặt dưới 5 site: chọn theo bảng Site lẻ.</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -828,7 +828,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Gói bao gồm</t>
+          <t>Chính sách gói</t>
         </is>
       </c>
     </row>
@@ -847,149 +847,143 @@
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Liên kết</t>
+          <t>Đặt dưới 5 site</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Mỗi bài đặt 02 liên kết về website của khách. Thuộc tính dofollow/nofollow do từng website xuất bản quyết định.</t>
+          <t>Cần ít hơn 5 site (ví dụ 2 site): đặt theo bảng Site lẻ, chọn đúng domain mong muốn, giá tính theo từng site.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Nội dung</t>
+          <t>Liên kết</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Miễn phí viết bài 900-1.200 từ, 3 hình ảnh (không gồm video), chỉnh sửa tối đa 3 lần. Anchor text và URL đích khách chốt trước khi gửi xuất bản, không đổi được sau khi đã gửi.</t>
+          <t>Mỗi bài đặt 02 liên kết về website của khách. Thuộc tính dofollow/nofollow do từng website xuất bản quyết định.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Chọn site</t>
+          <t>Nội dung</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Gói không chọn site theo chỉ định: hệ thống phân bổ site phù hợp chủ đề website của khách từ danh sách bên dưới. Các site là trang tổng hợp có tiểu mục liên quan, không chia theo ngành.</t>
+          <t>Áp dụng cho cả gói và site lẻ: miễn phí viết bài 900-1.200 từ, 3 hình ảnh (không gồm video), chỉnh sửa tối đa 3 lần. Anchor text và URL đích khách chốt trước khi gửi xuất bản, không đổi được sau khi đã gửi.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Thời gian</t>
+          <t>Chọn site trong gói</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Hoàn thiện 21-25 ngày kể từ khi triển khai, tuỳ thời gian chỉnh sửa và duyệt nội dung của mỗi bên. Khi đã duyệt xong, bài lên trong 1-2 ngày.</t>
+          <t>Gói không chọn site theo chỉ định: hệ thống phân bổ site phù hợp chủ đề website của khách từ danh sách 15 site. Các site là trang tổng hợp có tiểu mục liên quan, không chia theo ngành.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Bảo hành</t>
+          <t>Thời gian</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Bảo hành liên kết 03 tháng. Bài viết tồn tại theo vòng đời của site (đổi cấu trúc, sáp nhập hoặc ngừng hoạt động).</t>
+          <t>Hoàn thiện 21-25 ngày kể từ khi triển khai, tuỳ thời gian chỉnh sửa và duyệt nội dung của mỗi bên. Khi nội dung đã duyệt, bài lên trong 1-2 ngày.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Lĩnh vực không nhận</t>
+          <t>Bảo hành</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Tiền ảo, cho vay, casino và sản phẩm/dịch vụ không phù hợp chính sách của các website.</t>
+          <t>Bảo hành 03 tháng kể từ ngày bài lên: nếu bài viết bị gỡ hoặc mất trong thời gian này, DigicomVN yêu cầu đăng lại miễn phí.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Hoá đơn</t>
+          <t>Thời hạn bài viết</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
+          <t>Sau thời gian bảo hành, bài viết tiếp tục tồn tại cho đến khi site ngừng hoạt động, đổi cấu trúc hoặc sáp nhập với site khác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Lĩnh vực không nhận</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Tiền ảo, cho vay, casino và sản phẩm/dịch vụ không phù hợp chính sách của các website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Hoá đơn VAT</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
           <t>Dịch vụ đăng bài trên website nước ngoài nên đơn hàng này KHÔNG xuất được hoá đơn VAT.</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Danh sách 15 site trong hệ thống gói (phân bổ theo chủ đề, không chọn site)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>techbullion.com</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>itsreleased.com</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>usatimemagazine.co.uk</t>
+          <t>techbullion.com</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr"/>
@@ -1000,11 +994,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>namescastle.com</t>
+          <t>itsreleased.com</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr"/>
@@ -1015,11 +1009,11 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>publicistpaper.com</t>
+          <t>usatimemagazine.co.uk</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr"/>
@@ -1030,11 +1024,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>bignewsnetwork.com</t>
+          <t>namescastle.com</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr"/>
@@ -1045,11 +1039,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>bmtimes.co.uk</t>
+          <t>publicistpaper.com</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr"/>
@@ -1060,11 +1054,11 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>theinscribermag.com</t>
+          <t>bignewsnetwork.com</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr"/>
@@ -1075,11 +1069,11 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>timebusinessnews.com</t>
+          <t>bmtimes.co.uk</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr"/>
@@ -1090,11 +1084,11 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>businessnewstips.com</t>
+          <t>theinscribermag.com</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr"/>
@@ -1105,11 +1099,11 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>londondaily.news</t>
+          <t>timebusinessnews.com</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr"/>
@@ -1120,11 +1114,11 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>businesstomark.com</t>
+          <t>businessnewstips.com</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr"/>
@@ -1135,11 +1129,11 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>techbetime.com</t>
+          <t>londondaily.news</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr"/>
@@ -1150,11 +1144,11 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>techktimes.co.uk</t>
+          <t>businesstomark.com</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr"/>
@@ -1165,11 +1159,11 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>speromagazine.com</t>
+          <t>techbetime.com</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr"/>
@@ -1178,18 +1172,50 @@
       <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="4" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>techktimes.co.uk</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>speromagazine.com</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B19:G19"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="B14:G14"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="B13:G13"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="B18:G18"/>
     <mergeCell ref="B15:G15"/>
     <mergeCell ref="B11:G11"/>
   </mergeCells>
@@ -1204,7 +1230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1237,7 +1263,7 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Mỗi bài: 02 liên kết, nội dung miễn phí 900-1.200 từ, 3 hình ảnh, chỉnh sửa tối đa 3 lần. Site lẻ không áp dụng vào gói.</t>
+          <t>Mỗi bài: 02 liên kết, viết bài miễn phí 900-1.200 từ, 3 hình ảnh, sửa tối đa 3 lần, bảo hành 03 tháng, không xuất VAT. Chính sách đầy đủ ở cuối bảng.</t>
         </is>
       </c>
     </row>
@@ -3843,19 +3869,145 @@
       </c>
     </row>
     <row r="65"/>
-    <row r="66" ht="60" customHeight="1">
-      <c r="A66" s="6" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>Chính sách áp dụng cho site lẻ</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="34" customHeight="1">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>Số bài</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>Mỗi site 1 bài viết riêng. Ví dụ gói Starter = 5 site = 5 bài viết khác nhau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="34" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Đặt dưới 5 site</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Cần ít hơn 5 site (ví dụ 2 site): đặt theo bảng Site lẻ, chọn đúng domain mong muốn, giá tính theo từng site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="34" customHeight="1">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Liên kết</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Mỗi bài đặt 02 liên kết về website của khách. Thuộc tính dofollow/nofollow do từng website xuất bản quyết định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="34" customHeight="1">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Áp dụng cho cả gói và site lẻ: miễn phí viết bài 900-1.200 từ, 3 hình ảnh (không gồm video), chỉnh sửa tối đa 3 lần. Anchor text và URL đích khách chốt trước khi gửi xuất bản, không đổi được sau khi đã gửi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="34" customHeight="1">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Thời gian</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Hoàn thiện 21-25 ngày kể từ khi triển khai, tuỳ thời gian chỉnh sửa và duyệt nội dung của mỗi bên. Khi nội dung đã duyệt, bài lên trong 1-2 ngày.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="34" customHeight="1">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Bảo hành</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Bảo hành 03 tháng kể từ ngày bài lên: nếu bài viết bị gỡ hoặc mất trong thời gian này, DigicomVN yêu cầu đăng lại miễn phí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="34" customHeight="1">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Thời hạn bài viết</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Sau thời gian bảo hành, bài viết tiếp tục tồn tại cho đến khi site ngừng hoạt động, đổi cấu trúc hoặc sáp nhập với site khác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="34" customHeight="1">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>Lĩnh vực không nhận</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Tiền ảo, cho vay, casino và sản phẩm/dịch vụ không phù hợp chính sách của các website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="34" customHeight="1">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Hoá đơn VAT</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Dịch vụ đăng bài trên website nước ngoài nên đơn hàng này KHÔNG xuất được hoá đơn VAT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76"/>
+    <row r="77" ht="60" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
         <is>
           <t>Lưu ý khi chọn site lẻ: chỉ số DR và traffic ghi nhận tại thời điểm cập nhật, có thể biến động theo dữ liệu Ahrefs/Similarweb. Nên đánh giá site theo nhiều chỉ số (DR, traffic, mức liên quan chủ đề). Khi đặt nhiều site, nên đa dạng anchor text và URL đích. Một số site tải chậm do máy chủ đặt ở nước ngoài.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="14">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B72:J72"/>
+    <mergeCell ref="B67:J67"/>
+    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A4:J4"/>
+    <mergeCell ref="B71:J71"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B75:J75"/>
+    <mergeCell ref="B73:J73"/>
+    <mergeCell ref="B74:J74"/>
+    <mergeCell ref="B69:J69"/>
+    <mergeCell ref="B70:J70"/>
+    <mergeCell ref="B68:J68"/>
     <mergeCell ref="A66:J66"/>
-    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId1"/>
@@ -3927,7 +4079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4056,82 +4208,106 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Liên kết</t>
+          <t>Đặt dưới 5 site</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Mỗi bài đặt 02 liên kết về website của khách. Thuộc tính dofollow/nofollow do từng website xuất bản quyết định.</t>
+          <t>Cần ít hơn 5 site (ví dụ 2 site): đặt theo bảng Site lẻ, chọn đúng domain mong muốn, giá tính theo từng site.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Nội dung</t>
+          <t>Liên kết</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Miễn phí viết bài 900-1.200 từ, 3 hình ảnh (không gồm video), chỉnh sửa tối đa 3 lần. Anchor text và URL đích khách chốt trước khi gửi xuất bản, không đổi được sau khi đã gửi.</t>
+          <t>Mỗi bài đặt 02 liên kết về website của khách. Thuộc tính dofollow/nofollow do từng website xuất bản quyết định.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Chọn site</t>
+          <t>Nội dung</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Gói không chọn site theo chỉ định: hệ thống phân bổ site phù hợp chủ đề website của khách từ danh sách bên dưới. Các site là trang tổng hợp có tiểu mục liên quan, không chia theo ngành.</t>
+          <t>Áp dụng cho cả gói và site lẻ: miễn phí viết bài 900-1.200 từ, 3 hình ảnh (không gồm video), chỉnh sửa tối đa 3 lần. Anchor text và URL đích khách chốt trước khi gửi xuất bản, không đổi được sau khi đã gửi.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Thời gian</t>
+          <t>Chọn site trong gói</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Hoàn thiện 21-25 ngày kể từ khi triển khai, tuỳ thời gian chỉnh sửa và duyệt nội dung của mỗi bên. Khi đã duyệt xong, bài lên trong 1-2 ngày.</t>
+          <t>Gói không chọn site theo chỉ định: hệ thống phân bổ site phù hợp chủ đề website của khách từ danh sách 15 site. Các site là trang tổng hợp có tiểu mục liên quan, không chia theo ngành.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Bảo hành</t>
+          <t>Thời gian</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Bảo hành liên kết 03 tháng. Bài viết tồn tại theo vòng đời của site (đổi cấu trúc, sáp nhập hoặc ngừng hoạt động).</t>
+          <t>Hoàn thiện 21-25 ngày kể từ khi triển khai, tuỳ thời gian chỉnh sửa và duyệt nội dung của mỗi bên. Khi nội dung đã duyệt, bài lên trong 1-2 ngày.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Lĩnh vực không nhận</t>
+          <t>Bảo hành</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Tiền ảo, cho vay, casino và sản phẩm/dịch vụ không phù hợp chính sách của các website.</t>
+          <t>Bảo hành 03 tháng kể từ ngày bài lên: nếu bài viết bị gỡ hoặc mất trong thời gian này, DigicomVN yêu cầu đăng lại miễn phí.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Hoá đơn</t>
+          <t>Thời hạn bài viết</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Sau thời gian bảo hành, bài viết tiếp tục tồn tại cho đến khi site ngừng hoạt động, đổi cấu trúc hoặc sáp nhập với site khác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Lĩnh vực không nhận</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Tiền ảo, cho vay, casino và sản phẩm/dịch vụ không phù hợp chính sách của các website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hoá đơn VAT</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Dịch vụ đăng bài trên website nước ngoài nên đơn hàng này KHÔNG xuất được hoá đơn VAT.</t>
         </is>

</xml_diff>